<commit_message>
Task 1+2 complet: 714/720 lignes remplies (720 - 6 lignes n.d. sans source)
https://claude.ai/code/session_0159tTShW6o8QkMiD1mK29Qi
</commit_message>
<xml_diff>
--- a/work/source_v2.xlsx
+++ b/work/source_v2.xlsx
@@ -30101,7 +30101,7 @@
     <row r="639">
       <c r="A639" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B639" s="2" t="inlineStr">
@@ -30119,15 +30119,31 @@
           <t>Bitdeer Technologies</t>
         </is>
       </c>
-      <c r="F639" s="2" t="n"/>
-      <c r="G639" s="2" t="n"/>
-      <c r="H639" s="2" t="n"/>
-      <c r="I639" s="2" t="n"/>
+      <c r="F639" s="2" t="inlineStr">
+        <is>
+          <t>Mid cap 200M-1Md</t>
+        </is>
+      </c>
+      <c r="G639" s="2" t="inlineStr">
+        <is>
+          <t>USD 349.8 M</t>
+        </is>
+      </c>
+      <c r="H639" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I639" s="2" t="inlineStr">
+        <is>
+          <t>https://news.moomoo.com/notice/304320967/bitdeer-technologies-20-f-registration-statement-annual-report-transition-report</t>
+        </is>
+      </c>
     </row>
     <row r="640">
       <c r="A640" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Non</t>
         </is>
       </c>
       <c r="B640" s="2" t="inlineStr">
@@ -30145,15 +30161,31 @@
           <t>Bitmain Technologies</t>
         </is>
       </c>
-      <c r="F640" s="2" t="n"/>
-      <c r="G640" s="2" t="n"/>
-      <c r="H640" s="2" t="n"/>
-      <c r="I640" s="2" t="n"/>
+      <c r="F640" s="2" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="G640" s="2" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H640" s="2" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="I640" s="2" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
     </row>
     <row r="641">
       <c r="A641" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Non</t>
         </is>
       </c>
       <c r="B641" s="2" t="inlineStr">
@@ -30171,15 +30203,31 @@
           <t>MicroBT</t>
         </is>
       </c>
-      <c r="F641" s="2" t="n"/>
-      <c r="G641" s="2" t="n"/>
-      <c r="H641" s="2" t="n"/>
-      <c r="I641" s="2" t="n"/>
+      <c r="F641" s="2" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="G641" s="2" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H641" s="2" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="I641" s="2" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
     </row>
     <row r="642">
       <c r="A642" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B642" s="2" t="inlineStr">
@@ -30197,15 +30245,31 @@
           <t>Canaan Inc.</t>
         </is>
       </c>
-      <c r="F642" s="2" t="n"/>
-      <c r="G642" s="2" t="n"/>
-      <c r="H642" s="2" t="n"/>
-      <c r="I642" s="2" t="n"/>
+      <c r="F642" s="2" t="inlineStr">
+        <is>
+          <t>Mid cap 200M-1Md</t>
+        </is>
+      </c>
+      <c r="G642" s="2" t="inlineStr">
+        <is>
+          <t>USD 269.3 M</t>
+        </is>
+      </c>
+      <c r="H642" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I642" s="2" t="inlineStr">
+        <is>
+          <t>https://investor.canaan-creative.com/news-releases/news-release-details/canaan-inc-reports-unaudited-fourth-quarter-and-full-year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="643">
       <c r="A643" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B643" s="2" t="inlineStr">
@@ -30215,7 +30279,7 @@
       </c>
       <c r="C643" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>IA / Numérique</t>
         </is>
       </c>
       <c r="D643" s="2" t="inlineStr">
@@ -30223,15 +30287,31 @@
           <t>GMO Internet Group</t>
         </is>
       </c>
-      <c r="F643" s="2" t="n"/>
-      <c r="G643" s="2" t="n"/>
-      <c r="H643" s="2" t="n"/>
-      <c r="I643" s="2" t="n"/>
+      <c r="F643" s="2" t="inlineStr">
+        <is>
+          <t>Large cap / groupe &gt;1 Md</t>
+        </is>
+      </c>
+      <c r="G643" s="2" t="inlineStr">
+        <is>
+          <t>JPY 277.41 Md</t>
+        </is>
+      </c>
+      <c r="H643" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I643" s="2" t="inlineStr">
+        <is>
+          <t>https://stockanalysis.com/quote/otc/GMOYF/revenue/</t>
+        </is>
+      </c>
     </row>
     <row r="644">
       <c r="A644" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B644" s="2" t="inlineStr">
@@ -30241,7 +30321,7 @@
       </c>
       <c r="C644" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>IA / Numérique</t>
         </is>
       </c>
       <c r="D644" s="2" t="inlineStr">
@@ -30249,15 +30329,31 @@
           <t>SBI Holdings</t>
         </is>
       </c>
-      <c r="F644" s="2" t="n"/>
-      <c r="G644" s="2" t="n"/>
-      <c r="H644" s="2" t="n"/>
-      <c r="I644" s="2" t="n"/>
+      <c r="F644" s="2" t="inlineStr">
+        <is>
+          <t>Large cap / groupe &gt;1 Md</t>
+        </is>
+      </c>
+      <c r="G644" s="2" t="inlineStr">
+        <is>
+          <t>JPY 225.4 Md</t>
+        </is>
+      </c>
+      <c r="H644" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I644" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sbigroup.co.jp/english/investors/disclosure/presentation/pdf/250509presentations.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="645">
       <c r="A645" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B645" s="2" t="inlineStr">
@@ -30267,7 +30363,7 @@
       </c>
       <c r="C645" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Quantique</t>
         </is>
       </c>
       <c r="D645" s="2" t="inlineStr">
@@ -30275,15 +30371,31 @@
           <t>TSMC</t>
         </is>
       </c>
-      <c r="F645" s="2" t="n"/>
-      <c r="G645" s="2" t="n"/>
-      <c r="H645" s="2" t="n"/>
-      <c r="I645" s="2" t="n"/>
+      <c r="F645" s="2" t="inlineStr">
+        <is>
+          <t>Large cap / groupe &gt;1 Md</t>
+        </is>
+      </c>
+      <c r="G645" s="2" t="inlineStr">
+        <is>
+          <t>TWD 2 894 Md</t>
+        </is>
+      </c>
+      <c r="H645" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I645" s="2" t="inlineStr">
+        <is>
+          <t>https://investor.tsmc.com/static/annualReports/2024/english/index.html</t>
+        </is>
+      </c>
     </row>
     <row r="646">
       <c r="A646" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B646" s="2" t="inlineStr">
@@ -30293,7 +30405,7 @@
       </c>
       <c r="C646" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Quantique</t>
         </is>
       </c>
       <c r="D646" s="2" t="inlineStr">
@@ -30301,15 +30413,31 @@
           <t>MediaTek</t>
         </is>
       </c>
-      <c r="F646" s="2" t="n"/>
-      <c r="G646" s="2" t="n"/>
-      <c r="H646" s="2" t="n"/>
-      <c r="I646" s="2" t="n"/>
+      <c r="F646" s="2" t="inlineStr">
+        <is>
+          <t>Large cap / groupe &gt;1 Md</t>
+        </is>
+      </c>
+      <c r="G646" s="2" t="inlineStr">
+        <is>
+          <t>TWD 530.6 Md</t>
+        </is>
+      </c>
+      <c r="H646" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I646" s="2" t="inlineStr">
+        <is>
+          <t>https://stockanalysis.com/quote/tpe/2454/revenue/</t>
+        </is>
+      </c>
     </row>
     <row r="647">
       <c r="A647" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B647" s="2" t="inlineStr">
@@ -30319,7 +30447,7 @@
       </c>
       <c r="C647" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Quantique</t>
         </is>
       </c>
       <c r="D647" s="2" t="inlineStr">
@@ -30327,15 +30455,31 @@
           <t>Foxconn</t>
         </is>
       </c>
-      <c r="F647" s="2" t="n"/>
-      <c r="G647" s="2" t="n"/>
-      <c r="H647" s="2" t="n"/>
-      <c r="I647" s="2" t="n"/>
+      <c r="F647" s="2" t="inlineStr">
+        <is>
+          <t>Large cap / groupe &gt;1 Md</t>
+        </is>
+      </c>
+      <c r="G647" s="2" t="inlineStr">
+        <is>
+          <t>TWD 6 860 Md</t>
+        </is>
+      </c>
+      <c r="H647" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I647" s="2" t="inlineStr">
+        <is>
+          <t>https://www.foxconn.com/en-us/press-center/press-releases/latest-news/1554</t>
+        </is>
+      </c>
     </row>
     <row r="648">
       <c r="A648" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B648" s="2" t="inlineStr">
@@ -30345,7 +30489,7 @@
       </c>
       <c r="C648" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Quantique</t>
         </is>
       </c>
       <c r="D648" s="2" t="inlineStr">
@@ -30353,15 +30497,31 @@
           <t>Quanta Computer</t>
         </is>
       </c>
-      <c r="F648" s="2" t="n"/>
-      <c r="G648" s="2" t="n"/>
-      <c r="H648" s="2" t="n"/>
-      <c r="I648" s="2" t="n"/>
+      <c r="F648" s="2" t="inlineStr">
+        <is>
+          <t>Large cap / groupe &gt;1 Md</t>
+        </is>
+      </c>
+      <c r="G648" s="2" t="inlineStr">
+        <is>
+          <t>TWD 1 410 Md</t>
+        </is>
+      </c>
+      <c r="H648" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I648" s="2" t="inlineStr">
+        <is>
+          <t>https://stockanalysis.com/quote/tpe/2382/revenue/</t>
+        </is>
+      </c>
     </row>
     <row r="649">
       <c r="A649" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B649" s="2" t="inlineStr">
@@ -30371,7 +30531,7 @@
       </c>
       <c r="C649" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Quantique</t>
         </is>
       </c>
       <c r="D649" s="2" t="inlineStr">
@@ -30379,15 +30539,31 @@
           <t>Delta Electronics</t>
         </is>
       </c>
-      <c r="F649" s="2" t="n"/>
-      <c r="G649" s="2" t="n"/>
-      <c r="H649" s="2" t="n"/>
-      <c r="I649" s="2" t="n"/>
+      <c r="F649" s="2" t="inlineStr">
+        <is>
+          <t>Large cap / groupe &gt;1 Md</t>
+        </is>
+      </c>
+      <c r="G649" s="2" t="inlineStr">
+        <is>
+          <t>TWD 421.1 Md</t>
+        </is>
+      </c>
+      <c r="H649" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I649" s="2" t="inlineStr">
+        <is>
+          <t>https://filecenter.deltaww.com/ir/download/financial_report/Q42024_eng_Consolidated%20Financial%20Report.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="650">
       <c r="A650" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B650" s="2" t="inlineStr">
@@ -30397,7 +30573,7 @@
       </c>
       <c r="C650" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Quantique</t>
         </is>
       </c>
       <c r="D650" s="2" t="inlineStr">
@@ -30405,15 +30581,31 @@
           <t>Samsung Electronics</t>
         </is>
       </c>
-      <c r="F650" s="2" t="n"/>
-      <c r="G650" s="2" t="n"/>
-      <c r="H650" s="2" t="n"/>
-      <c r="I650" s="2" t="n"/>
+      <c r="F650" s="2" t="inlineStr">
+        <is>
+          <t>Large cap / groupe &gt;1 Md</t>
+        </is>
+      </c>
+      <c r="G650" s="2" t="inlineStr">
+        <is>
+          <t>KRW 300 875 Md</t>
+        </is>
+      </c>
+      <c r="H650" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I650" s="2" t="inlineStr">
+        <is>
+          <t>https://news.samsung.com/global/samsung-electronics-announces-fourth-quarter-and-fy-2024-results</t>
+        </is>
+      </c>
     </row>
     <row r="651">
       <c r="A651" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B651" s="2" t="inlineStr">
@@ -30423,7 +30615,7 @@
       </c>
       <c r="C651" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Quantique</t>
         </is>
       </c>
       <c r="D651" s="2" t="inlineStr">
@@ -30431,15 +30623,31 @@
           <t>SK hynix</t>
         </is>
       </c>
-      <c r="F651" s="2" t="n"/>
-      <c r="G651" s="2" t="n"/>
-      <c r="H651" s="2" t="n"/>
-      <c r="I651" s="2" t="n"/>
+      <c r="F651" s="2" t="inlineStr">
+        <is>
+          <t>Large cap / groupe &gt;1 Md</t>
+        </is>
+      </c>
+      <c r="G651" s="2" t="inlineStr">
+        <is>
+          <t>KRW 66 193 Md</t>
+        </is>
+      </c>
+      <c r="H651" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I651" s="2" t="inlineStr">
+        <is>
+          <t>https://news.skhynix.com/sk-hynix-announces-4q24-financial-results/</t>
+        </is>
+      </c>
     </row>
     <row r="652">
       <c r="A652" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B652" s="2" t="inlineStr">
@@ -30449,7 +30657,7 @@
       </c>
       <c r="C652" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Énergie</t>
         </is>
       </c>
       <c r="D652" s="2" t="inlineStr">
@@ -30457,15 +30665,31 @@
           <t>CLP Holdings</t>
         </is>
       </c>
-      <c r="F652" s="2" t="n"/>
-      <c r="G652" s="2" t="n"/>
-      <c r="H652" s="2" t="n"/>
-      <c r="I652" s="2" t="n"/>
+      <c r="F652" s="2" t="inlineStr">
+        <is>
+          <t>Large cap / groupe &gt;1 Md</t>
+        </is>
+      </c>
+      <c r="G652" s="2" t="inlineStr">
+        <is>
+          <t>HKD 91.0 Md</t>
+        </is>
+      </c>
+      <c r="H652" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I652" s="2" t="inlineStr">
+        <is>
+          <t>https://annualreport.clpgroup.com/AR2024/Snapshot/en/financial-performance.html</t>
+        </is>
+      </c>
     </row>
     <row r="653">
       <c r="A653" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B653" s="2" t="inlineStr">
@@ -30475,7 +30699,7 @@
       </c>
       <c r="C653" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Énergie</t>
         </is>
       </c>
       <c r="D653" s="2" t="inlineStr">
@@ -30483,10 +30707,26 @@
           <t>KEPCO</t>
         </is>
       </c>
-      <c r="F653" s="2" t="n"/>
-      <c r="G653" s="2" t="n"/>
-      <c r="H653" s="2" t="n"/>
-      <c r="I653" s="2" t="n"/>
+      <c r="F653" s="2" t="inlineStr">
+        <is>
+          <t>Large cap / groupe &gt;1 Md</t>
+        </is>
+      </c>
+      <c r="G653" s="2" t="inlineStr">
+        <is>
+          <t>KRW 94 001 Md</t>
+        </is>
+      </c>
+      <c r="H653" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I653" s="2" t="inlineStr">
+        <is>
+          <t>https://cm.asiae.co.kr/en/article/2025022814314291606</t>
+        </is>
+      </c>
     </row>
     <row r="654">
       <c r="A654" s="5" t="inlineStr">
@@ -33641,7 +33881,7 @@
     <row r="729">
       <c r="A729" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B729" s="2" t="inlineStr">
@@ -33651,7 +33891,7 @@
       </c>
       <c r="C729" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Énergie</t>
         </is>
       </c>
       <c r="D729" s="2" t="inlineStr">
@@ -33659,15 +33899,31 @@
           <t>Eletrobras</t>
         </is>
       </c>
-      <c r="F729" s="2" t="n"/>
-      <c r="G729" s="2" t="n"/>
-      <c r="H729" s="2" t="n"/>
-      <c r="I729" s="2" t="n"/>
+      <c r="F729" s="2" t="inlineStr">
+        <is>
+          <t>Large cap / groupe &gt;1 Md</t>
+        </is>
+      </c>
+      <c r="G729" s="2" t="inlineStr">
+        <is>
+          <t>BRL 40.18 Md</t>
+        </is>
+      </c>
+      <c r="H729" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I729" s="2" t="inlineStr">
+        <is>
+          <t>https://www.macrotrends.net/stocks/charts/EBR.B/eletrobras/revenue</t>
+        </is>
+      </c>
     </row>
     <row r="730">
       <c r="A730" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B730" s="2" t="inlineStr">
@@ -33677,7 +33933,7 @@
       </c>
       <c r="C730" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Énergie</t>
         </is>
       </c>
       <c r="D730" s="2" t="inlineStr">
@@ -33685,15 +33941,31 @@
           <t>Cemig</t>
         </is>
       </c>
-      <c r="F730" s="2" t="n"/>
-      <c r="G730" s="2" t="n"/>
-      <c r="H730" s="2" t="n"/>
-      <c r="I730" s="2" t="n"/>
+      <c r="F730" s="2" t="inlineStr">
+        <is>
+          <t>Large cap / groupe &gt;1 Md</t>
+        </is>
+      </c>
+      <c r="G730" s="2" t="inlineStr">
+        <is>
+          <t>BRL 39.8 Md</t>
+        </is>
+      </c>
+      <c r="H730" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I730" s="2" t="inlineStr">
+        <is>
+          <t>https://ri.cemig.com.br/en</t>
+        </is>
+      </c>
     </row>
     <row r="731">
       <c r="A731" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B731" s="2" t="inlineStr">
@@ -33703,7 +33975,7 @@
       </c>
       <c r="C731" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Énergie</t>
         </is>
       </c>
       <c r="D731" s="2" t="inlineStr">
@@ -33711,15 +33983,31 @@
           <t>Copel</t>
         </is>
       </c>
-      <c r="F731" s="2" t="n"/>
-      <c r="G731" s="2" t="n"/>
-      <c r="H731" s="2" t="n"/>
-      <c r="I731" s="2" t="n"/>
+      <c r="F731" s="2" t="inlineStr">
+        <is>
+          <t>Large cap / groupe &gt;1 Md</t>
+        </is>
+      </c>
+      <c r="G731" s="2" t="inlineStr">
+        <is>
+          <t>USD 4.2 Md</t>
+        </is>
+      </c>
+      <c r="H731" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I731" s="2" t="inlineStr">
+        <is>
+          <t>https://www.macrotrends.net/stocks/charts/ELP/companhia-paranaense-de-energia-copel/revenue</t>
+        </is>
+      </c>
     </row>
     <row r="732">
       <c r="A732" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B732" s="2" t="inlineStr">
@@ -33729,7 +34017,7 @@
       </c>
       <c r="C732" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Énergie</t>
         </is>
       </c>
       <c r="D732" s="2" t="inlineStr">
@@ -33737,15 +34025,31 @@
           <t>Engie Brasil Energia</t>
         </is>
       </c>
-      <c r="F732" s="2" t="n"/>
-      <c r="G732" s="2" t="n"/>
-      <c r="H732" s="2" t="n"/>
-      <c r="I732" s="2" t="n"/>
+      <c r="F732" s="2" t="inlineStr">
+        <is>
+          <t>Large cap / groupe &gt;1 Md</t>
+        </is>
+      </c>
+      <c r="G732" s="2" t="inlineStr">
+        <is>
+          <t>BRL 11.22 Md</t>
+        </is>
+      </c>
+      <c r="H732" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I732" s="2" t="inlineStr">
+        <is>
+          <t>https://stockanalysis.com/quote/bvmf/EGIE3/revenue/</t>
+        </is>
+      </c>
     </row>
     <row r="733">
       <c r="A733" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B733" s="2" t="inlineStr">
@@ -33755,7 +34059,7 @@
       </c>
       <c r="C733" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Énergie</t>
         </is>
       </c>
       <c r="D733" s="2" t="inlineStr">
@@ -33763,15 +34067,31 @@
           <t>AES Brasil</t>
         </is>
       </c>
-      <c r="F733" s="2" t="n"/>
-      <c r="G733" s="2" t="n"/>
-      <c r="H733" s="2" t="n"/>
-      <c r="I733" s="2" t="n"/>
+      <c r="F733" s="2" t="inlineStr">
+        <is>
+          <t>Mid cap 200M-1Md</t>
+        </is>
+      </c>
+      <c r="G733" s="2" t="inlineStr">
+        <is>
+          <t>BRL 3.78 Md</t>
+        </is>
+      </c>
+      <c r="H733" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I733" s="2" t="inlineStr">
+        <is>
+          <t>https://stockanalysis.com/quote/bvmf/AESB3/revenue/</t>
+        </is>
+      </c>
     </row>
     <row r="734">
       <c r="A734" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B734" s="2" t="inlineStr">
@@ -33781,7 +34101,7 @@
       </c>
       <c r="C734" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Énergie</t>
         </is>
       </c>
       <c r="D734" s="2" t="inlineStr">
@@ -33789,15 +34109,31 @@
           <t>Eneva</t>
         </is>
       </c>
-      <c r="F734" s="2" t="n"/>
-      <c r="G734" s="2" t="n"/>
-      <c r="H734" s="2" t="n"/>
-      <c r="I734" s="2" t="n"/>
+      <c r="F734" s="2" t="inlineStr">
+        <is>
+          <t>Large cap / groupe &gt;1 Md</t>
+        </is>
+      </c>
+      <c r="G734" s="2" t="inlineStr">
+        <is>
+          <t>BRL 11.39 Md</t>
+        </is>
+      </c>
+      <c r="H734" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I734" s="2" t="inlineStr">
+        <is>
+          <t>https://stockanalysis.com/quote/bvmf/ENEV3/</t>
+        </is>
+      </c>
     </row>
     <row r="735">
       <c r="A735" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B735" s="2" t="inlineStr">
@@ -33807,7 +34143,7 @@
       </c>
       <c r="C735" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Énergie</t>
         </is>
       </c>
       <c r="D735" s="2" t="inlineStr">
@@ -33815,15 +34151,31 @@
           <t>CPFL Energia</t>
         </is>
       </c>
-      <c r="F735" s="2" t="n"/>
-      <c r="G735" s="2" t="n"/>
-      <c r="H735" s="2" t="n"/>
-      <c r="I735" s="2" t="n"/>
+      <c r="F735" s="2" t="inlineStr">
+        <is>
+          <t>Large cap / groupe &gt;1 Md</t>
+        </is>
+      </c>
+      <c r="G735" s="2" t="inlineStr">
+        <is>
+          <t>BRL 42.63 Md</t>
+        </is>
+      </c>
+      <c r="H735" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I735" s="2" t="inlineStr">
+        <is>
+          <t>https://companiesmarketcap.com/cpfl-energia/revenue/</t>
+        </is>
+      </c>
     </row>
     <row r="736">
       <c r="A736" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B736" s="2" t="inlineStr">
@@ -33833,7 +34185,7 @@
       </c>
       <c r="C736" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Énergie</t>
         </is>
       </c>
       <c r="D736" s="2" t="inlineStr">
@@ -33841,15 +34193,31 @@
           <t>Enel Américas</t>
         </is>
       </c>
-      <c r="F736" s="2" t="n"/>
-      <c r="G736" s="2" t="n"/>
-      <c r="H736" s="2" t="n"/>
-      <c r="I736" s="2" t="n"/>
+      <c r="F736" s="2" t="inlineStr">
+        <is>
+          <t>Large cap / groupe &gt;1 Md</t>
+        </is>
+      </c>
+      <c r="G736" s="2" t="inlineStr">
+        <is>
+          <t>USD 12.61 Md</t>
+        </is>
+      </c>
+      <c r="H736" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I736" s="2" t="inlineStr">
+        <is>
+          <t>https://companiesmarketcap.com/enel-americas/revenue/</t>
+        </is>
+      </c>
     </row>
     <row r="737">
       <c r="A737" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B737" s="2" t="inlineStr">
@@ -33859,7 +34227,7 @@
       </c>
       <c r="C737" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Énergie</t>
         </is>
       </c>
       <c r="D737" s="2" t="inlineStr">
@@ -33867,15 +34235,31 @@
           <t>Colbún</t>
         </is>
       </c>
-      <c r="F737" s="2" t="n"/>
-      <c r="G737" s="2" t="n"/>
-      <c r="H737" s="2" t="n"/>
-      <c r="I737" s="2" t="n"/>
+      <c r="F737" s="2" t="inlineStr">
+        <is>
+          <t>Mid cap 200M-1Md</t>
+        </is>
+      </c>
+      <c r="G737" s="2" t="inlineStr">
+        <is>
+          <t>USD 1 576 M</t>
+        </is>
+      </c>
+      <c r="H737" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I737" s="2" t="inlineStr">
+        <is>
+          <t>https://www.colbun.cl/home/2025/01/29/colbun-cierra-2024-con-ebitda-de-us642-4-millones</t>
+        </is>
+      </c>
     </row>
     <row r="738">
       <c r="A738" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B738" s="2" t="inlineStr">
@@ -33885,7 +34269,7 @@
       </c>
       <c r="C738" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Énergie</t>
         </is>
       </c>
       <c r="D738" s="2" t="inlineStr">
@@ -33893,15 +34277,31 @@
           <t>Enel Chile</t>
         </is>
       </c>
-      <c r="F738" s="2" t="n"/>
-      <c r="G738" s="2" t="n"/>
-      <c r="H738" s="2" t="n"/>
-      <c r="I738" s="2" t="n"/>
+      <c r="F738" s="2" t="inlineStr">
+        <is>
+          <t>Large cap / groupe &gt;1 Md</t>
+        </is>
+      </c>
+      <c r="G738" s="2" t="inlineStr">
+        <is>
+          <t>USD 4.22 Md</t>
+        </is>
+      </c>
+      <c r="H738" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I738" s="2" t="inlineStr">
+        <is>
+          <t>https://companiesmarketcap.com/enel-chile/revenue/</t>
+        </is>
+      </c>
     </row>
     <row r="739">
       <c r="A739" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B739" s="2" t="inlineStr">
@@ -33911,7 +34311,7 @@
       </c>
       <c r="C739" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Énergie</t>
         </is>
       </c>
       <c r="D739" s="2" t="inlineStr">
@@ -33919,15 +34319,31 @@
           <t>ISA</t>
         </is>
       </c>
-      <c r="F739" s="2" t="n"/>
-      <c r="G739" s="2" t="n"/>
-      <c r="H739" s="2" t="n"/>
-      <c r="I739" s="2" t="n"/>
+      <c r="F739" s="2" t="inlineStr">
+        <is>
+          <t>Large cap / groupe &gt;1 Md</t>
+        </is>
+      </c>
+      <c r="G739" s="2" t="inlineStr">
+        <is>
+          <t>COP 14.74 T</t>
+        </is>
+      </c>
+      <c r="H739" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I739" s="2" t="inlineStr">
+        <is>
+          <t>https://stockanalysis.com/quote/bvc/ISA/revenue/</t>
+        </is>
+      </c>
     </row>
     <row r="740">
       <c r="A740" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B740" s="2" t="inlineStr">
@@ -33937,7 +34353,7 @@
       </c>
       <c r="C740" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Énergie</t>
         </is>
       </c>
       <c r="D740" s="2" t="inlineStr">
@@ -33945,15 +34361,31 @@
           <t>Grupo Energía Bogotá</t>
         </is>
       </c>
-      <c r="F740" s="2" t="n"/>
-      <c r="G740" s="2" t="n"/>
-      <c r="H740" s="2" t="n"/>
-      <c r="I740" s="2" t="n"/>
+      <c r="F740" s="2" t="inlineStr">
+        <is>
+          <t>Large cap / groupe &gt;1 Md</t>
+        </is>
+      </c>
+      <c r="G740" s="2" t="inlineStr">
+        <is>
+          <t>COP 7 972 Md</t>
+        </is>
+      </c>
+      <c r="H740" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I740" s="2" t="inlineStr">
+        <is>
+          <t>https://www.valoraanalitik.com/grupo-energia-bogota-cerro-2024-con-ingresos-de-8-billones-y-un-ebitda-ajustado-de-51-billones/</t>
+        </is>
+      </c>
     </row>
     <row r="741">
       <c r="A741" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B741" s="2" t="inlineStr">
@@ -33963,7 +34395,7 @@
       </c>
       <c r="C741" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Énergie</t>
         </is>
       </c>
       <c r="D741" s="2" t="inlineStr">
@@ -33971,15 +34403,31 @@
           <t>CFE</t>
         </is>
       </c>
-      <c r="F741" s="2" t="n"/>
-      <c r="G741" s="2" t="n"/>
-      <c r="H741" s="2" t="n"/>
-      <c r="I741" s="2" t="n"/>
+      <c r="F741" s="2" t="inlineStr">
+        <is>
+          <t>Large cap / groupe &gt;1 Md</t>
+        </is>
+      </c>
+      <c r="G741" s="2" t="inlineStr">
+        <is>
+          <t>MXN 667 Md</t>
+        </is>
+      </c>
+      <c r="H741" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I741" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cfe.gob.mx/finanzas/financial-economic-information/Quarterly%20Investor%20Presentations%20Doc/2024/120325_4T24_versi%C3%B3n%20ingl%C3%A9s_VFF.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="742">
       <c r="A742" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B742" s="2" t="inlineStr">
@@ -33989,7 +34437,7 @@
       </c>
       <c r="C742" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Énergie</t>
         </is>
       </c>
       <c r="D742" s="2" t="inlineStr">
@@ -33997,15 +34445,31 @@
           <t>Pampa Energía</t>
         </is>
       </c>
-      <c r="F742" s="2" t="n"/>
-      <c r="G742" s="2" t="n"/>
-      <c r="H742" s="2" t="n"/>
-      <c r="I742" s="2" t="n"/>
+      <c r="F742" s="2" t="inlineStr">
+        <is>
+          <t>Mid cap 200M-1Md</t>
+        </is>
+      </c>
+      <c r="G742" s="2" t="inlineStr">
+        <is>
+          <t>USD 1 876 M</t>
+        </is>
+      </c>
+      <c r="H742" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I742" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/0001469395/000129281425000808/ex99-1.htm</t>
+        </is>
+      </c>
     </row>
     <row r="743">
       <c r="A743" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B743" s="2" t="inlineStr">
@@ -34015,7 +34479,7 @@
       </c>
       <c r="C743" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Énergie</t>
         </is>
       </c>
       <c r="D743" s="2" t="inlineStr">
@@ -34023,10 +34487,26 @@
           <t>Pan American Energy</t>
         </is>
       </c>
-      <c r="F743" s="2" t="n"/>
-      <c r="G743" s="2" t="n"/>
-      <c r="H743" s="2" t="n"/>
-      <c r="I743" s="2" t="n"/>
+      <c r="F743" s="2" t="inlineStr">
+        <is>
+          <t>Large cap / groupe &gt;1 Md</t>
+        </is>
+      </c>
+      <c r="G743" s="2" t="inlineStr">
+        <is>
+          <t>USD 6.2 Md</t>
+        </is>
+      </c>
+      <c r="H743" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I743" s="2" t="inlineStr">
+        <is>
+          <t>https://www.zoominfo.com/c/pan-american-energy-llc/347331489</t>
+        </is>
+      </c>
     </row>
     <row r="744">
       <c r="A744" s="5" t="inlineStr">
@@ -37181,7 +37661,7 @@
     <row r="819">
       <c r="A819" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B819" s="2" t="inlineStr">
@@ -37191,7 +37671,7 @@
       </c>
       <c r="C819" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Énergie</t>
         </is>
       </c>
       <c r="D819" s="2" t="inlineStr">
@@ -37199,15 +37679,31 @@
           <t>KenGen</t>
         </is>
       </c>
-      <c r="F819" s="2" t="n"/>
-      <c r="G819" s="2" t="n"/>
-      <c r="H819" s="2" t="n"/>
-      <c r="I819" s="2" t="n"/>
+      <c r="F819" s="2" t="inlineStr">
+        <is>
+          <t>Mid cap 200M-1Md</t>
+        </is>
+      </c>
+      <c r="G819" s="2" t="inlineStr">
+        <is>
+          <t>KES 56.3 Md</t>
+        </is>
+      </c>
+      <c r="H819" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I819" s="2" t="inlineStr">
+        <is>
+          <t>https://kenyanwallstreet.com/kengens-profits-surge-35-5-to-kes-6-8-billion</t>
+        </is>
+      </c>
     </row>
     <row r="820">
       <c r="A820" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B820" s="2" t="inlineStr">
@@ -37217,7 +37713,7 @@
       </c>
       <c r="C820" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Énergie</t>
         </is>
       </c>
       <c r="D820" s="2" t="inlineStr">
@@ -37225,15 +37721,31 @@
           <t>Eskom</t>
         </is>
       </c>
-      <c r="F820" s="2" t="n"/>
-      <c r="G820" s="2" t="n"/>
-      <c r="H820" s="2" t="n"/>
-      <c r="I820" s="2" t="n"/>
+      <c r="F820" s="2" t="inlineStr">
+        <is>
+          <t>Large cap / groupe &gt;1 Md</t>
+        </is>
+      </c>
+      <c r="G820" s="2" t="inlineStr">
+        <is>
+          <t>ZAR 295.8 Md</t>
+        </is>
+      </c>
+      <c r="H820" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I820" s="2" t="inlineStr">
+        <is>
+          <t>https://www.eskom.co.za/wp-content/uploads/2024/12/Eskom-results-presentation-2024.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="821">
       <c r="A821" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B821" s="2" t="inlineStr">
@@ -37243,7 +37755,7 @@
       </c>
       <c r="C821" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Quantique</t>
         </is>
       </c>
       <c r="D821" s="2" t="inlineStr">
@@ -37251,15 +37763,31 @@
           <t>OCP Group</t>
         </is>
       </c>
-      <c r="F821" s="2" t="n"/>
-      <c r="G821" s="2" t="n"/>
-      <c r="H821" s="2" t="n"/>
-      <c r="I821" s="2" t="n"/>
+      <c r="F821" s="2" t="inlineStr">
+        <is>
+          <t>Large cap / groupe &gt;1 Md</t>
+        </is>
+      </c>
+      <c r="G821" s="2" t="inlineStr">
+        <is>
+          <t>USD 9.76 Md</t>
+        </is>
+      </c>
+      <c r="H821" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I821" s="2" t="inlineStr">
+        <is>
+          <t>https://news.frontierafricareports.com/article/ocp-reports-solid-performance-in-2024-revenues-rea</t>
+        </is>
+      </c>
     </row>
     <row r="822">
       <c r="A822" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B822" s="2" t="inlineStr">
@@ -37269,7 +37797,7 @@
       </c>
       <c r="C822" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Énergie</t>
         </is>
       </c>
       <c r="D822" s="2" t="inlineStr">
@@ -37277,15 +37805,31 @@
           <t>Sonatrach</t>
         </is>
       </c>
-      <c r="F822" s="2" t="n"/>
-      <c r="G822" s="2" t="n"/>
-      <c r="H822" s="2" t="n"/>
-      <c r="I822" s="2" t="n"/>
+      <c r="F822" s="2" t="inlineStr">
+        <is>
+          <t>Large cap / groupe &gt;1 Md</t>
+        </is>
+      </c>
+      <c r="G822" s="2" t="inlineStr">
+        <is>
+          <t>USD 45 Md</t>
+        </is>
+      </c>
+      <c r="H822" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I822" s="2" t="inlineStr">
+        <is>
+          <t>https://sonatrach.com/wp-content/uploads/2025/12/RA_2024_EN_-08-dec.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="823">
       <c r="A823" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B823" s="2" t="inlineStr">
@@ -37295,7 +37839,7 @@
       </c>
       <c r="C823" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Énergie</t>
         </is>
       </c>
       <c r="D823" s="2" t="inlineStr">
@@ -37303,15 +37847,31 @@
           <t>Sasol</t>
         </is>
       </c>
-      <c r="F823" s="2" t="n"/>
-      <c r="G823" s="2" t="n"/>
-      <c r="H823" s="2" t="n"/>
-      <c r="I823" s="2" t="n"/>
+      <c r="F823" s="2" t="inlineStr">
+        <is>
+          <t>Large cap / groupe &gt;1 Md</t>
+        </is>
+      </c>
+      <c r="G823" s="2" t="inlineStr">
+        <is>
+          <t>ZAR 275.1 Md</t>
+        </is>
+      </c>
+      <c r="H823" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I823" s="2" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/sasol-limited-audited-financial-results-for-the-year-ended-30-june-2024-302226150.html</t>
+        </is>
+      </c>
     </row>
     <row r="824">
       <c r="A824" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B824" s="2" t="inlineStr">
@@ -37321,7 +37881,7 @@
       </c>
       <c r="C824" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Quantique</t>
         </is>
       </c>
       <c r="D824" s="2" t="inlineStr">
@@ -37329,15 +37889,31 @@
           <t>Exxaro Resources</t>
         </is>
       </c>
-      <c r="F824" s="2" t="n"/>
-      <c r="G824" s="2" t="n"/>
-      <c r="H824" s="2" t="n"/>
-      <c r="I824" s="2" t="n"/>
+      <c r="F824" s="2" t="inlineStr">
+        <is>
+          <t>Large cap / groupe &gt;1 Md</t>
+        </is>
+      </c>
+      <c r="G824" s="2" t="inlineStr">
+        <is>
+          <t>USD 2.17 Md</t>
+        </is>
+      </c>
+      <c r="H824" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I824" s="2" t="inlineStr">
+        <is>
+          <t>https://investor.exxaro.com/financialresults/annual-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="825">
       <c r="A825" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B825" s="2" t="inlineStr">
@@ -37347,7 +37923,7 @@
       </c>
       <c r="C825" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Quantique</t>
         </is>
       </c>
       <c r="D825" s="2" t="inlineStr">
@@ -37355,15 +37931,31 @@
           <t>Gold Fields</t>
         </is>
       </c>
-      <c r="F825" s="2" t="n"/>
-      <c r="G825" s="2" t="n"/>
-      <c r="H825" s="2" t="n"/>
-      <c r="I825" s="2" t="n"/>
+      <c r="F825" s="2" t="inlineStr">
+        <is>
+          <t>Large cap / groupe &gt;1 Md</t>
+        </is>
+      </c>
+      <c r="G825" s="2" t="inlineStr">
+        <is>
+          <t>USD 5 202 M</t>
+        </is>
+      </c>
+      <c r="H825" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I825" s="2" t="inlineStr">
+        <is>
+          <t>https://www.goldfields.com/reports/q4-2025/revenue.php</t>
+        </is>
+      </c>
     </row>
     <row r="826">
       <c r="A826" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B826" s="2" t="inlineStr">
@@ -37373,7 +37965,7 @@
       </c>
       <c r="C826" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Quantique</t>
         </is>
       </c>
       <c r="D826" s="2" t="inlineStr">
@@ -37381,15 +37973,31 @@
           <t>Sibanye-Stillwater</t>
         </is>
       </c>
-      <c r="F826" s="2" t="n"/>
-      <c r="G826" s="2" t="n"/>
-      <c r="H826" s="2" t="n"/>
-      <c r="I826" s="2" t="n"/>
+      <c r="F826" s="2" t="inlineStr">
+        <is>
+          <t>Large cap / groupe &gt;1 Md</t>
+        </is>
+      </c>
+      <c r="G826" s="2" t="inlineStr">
+        <is>
+          <t>ZAR 56.9 Md</t>
+        </is>
+      </c>
+      <c r="H826" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I826" s="2" t="inlineStr">
+        <is>
+          <t>https://reports.sibanyestillwater.com/2024/</t>
+        </is>
+      </c>
     </row>
     <row r="827">
       <c r="A827" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B827" s="2" t="inlineStr">
@@ -37399,7 +38007,7 @@
       </c>
       <c r="C827" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Quantique</t>
         </is>
       </c>
       <c r="D827" s="2" t="inlineStr">
@@ -37407,15 +38015,31 @@
           <t>Impala Platinum</t>
         </is>
       </c>
-      <c r="F827" s="2" t="n"/>
-      <c r="G827" s="2" t="n"/>
-      <c r="H827" s="2" t="n"/>
-      <c r="I827" s="2" t="n"/>
+      <c r="F827" s="2" t="inlineStr">
+        <is>
+          <t>Large cap / groupe &gt;1 Md</t>
+        </is>
+      </c>
+      <c r="G827" s="2" t="inlineStr">
+        <is>
+          <t>ZAR 86.4 Md</t>
+        </is>
+      </c>
+      <c r="H827" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I827" s="2" t="inlineStr">
+        <is>
+          <t>https://stockanalysis.com/quote/otc/IMPUY/revenue/</t>
+        </is>
+      </c>
     </row>
     <row r="828">
       <c r="A828" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B828" s="2" t="inlineStr">
@@ -37425,7 +38049,7 @@
       </c>
       <c r="C828" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Quantique</t>
         </is>
       </c>
       <c r="D828" s="2" t="inlineStr">
@@ -37433,15 +38057,31 @@
           <t>Harmony Gold</t>
         </is>
       </c>
-      <c r="F828" s="2" t="n"/>
-      <c r="G828" s="2" t="n"/>
-      <c r="H828" s="2" t="n"/>
-      <c r="I828" s="2" t="n"/>
+      <c r="F828" s="2" t="inlineStr">
+        <is>
+          <t>Large cap / groupe &gt;1 Md</t>
+        </is>
+      </c>
+      <c r="G828" s="2" t="inlineStr">
+        <is>
+          <t>USD 3 282 M</t>
+        </is>
+      </c>
+      <c r="H828" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I828" s="2" t="inlineStr">
+        <is>
+          <t>https://www.nasdaq.com/articles/harmony-gold-minings-earnings-and-revenues-increase-fy24</t>
+        </is>
+      </c>
     </row>
     <row r="829">
       <c r="A829" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B829" s="2" t="inlineStr">
@@ -37451,7 +38091,7 @@
       </c>
       <c r="C829" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Quantique</t>
         </is>
       </c>
       <c r="D829" s="2" t="inlineStr">
@@ -37459,15 +38099,31 @@
           <t>Kumba Iron Ore</t>
         </is>
       </c>
-      <c r="F829" s="2" t="n"/>
-      <c r="G829" s="2" t="n"/>
-      <c r="H829" s="2" t="n"/>
-      <c r="I829" s="2" t="n"/>
+      <c r="F829" s="2" t="inlineStr">
+        <is>
+          <t>Large cap / groupe &gt;1 Md</t>
+        </is>
+      </c>
+      <c r="G829" s="2" t="inlineStr">
+        <is>
+          <t>ZAR 70.1 Md</t>
+        </is>
+      </c>
+      <c r="H829" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I829" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rttnews.com/3623064/kumba-iron-ore-fy-profit-slips-but-revenue-rises.aspx</t>
+        </is>
+      </c>
     </row>
     <row r="830">
       <c r="A830" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Non</t>
         </is>
       </c>
       <c r="B830" s="2" t="inlineStr">
@@ -37477,7 +38133,7 @@
       </c>
       <c r="C830" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Énergie</t>
         </is>
       </c>
       <c r="D830" s="2" t="inlineStr">
@@ -37485,15 +38141,31 @@
           <t>Egbin Power</t>
         </is>
       </c>
-      <c r="F830" s="2" t="n"/>
-      <c r="G830" s="2" t="n"/>
-      <c r="H830" s="2" t="n"/>
-      <c r="I830" s="2" t="n"/>
+      <c r="F830" s="2" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="G830" s="2" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H830" s="2" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="I830" s="2" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
     </row>
     <row r="831" ht="24" customHeight="1">
       <c r="A831" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Non</t>
         </is>
       </c>
       <c r="B831" s="2" t="inlineStr">
@@ -37503,7 +38175,7 @@
       </c>
       <c r="C831" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Énergie</t>
         </is>
       </c>
       <c r="D831" s="2" t="inlineStr">
@@ -37511,15 +38183,31 @@
           <t>Egyptian Electricity Holding</t>
         </is>
       </c>
-      <c r="F831" s="2" t="n"/>
-      <c r="G831" s="2" t="n"/>
-      <c r="H831" s="2" t="n"/>
-      <c r="I831" s="2" t="n"/>
+      <c r="F831" s="2" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="G831" s="2" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H831" s="2" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="I831" s="2" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
     </row>
     <row r="832">
       <c r="A832" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Non</t>
         </is>
       </c>
       <c r="B832" s="2" t="inlineStr">
@@ -37529,7 +38217,7 @@
       </c>
       <c r="C832" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Énergie</t>
         </is>
       </c>
       <c r="D832" s="2" t="inlineStr">
@@ -37537,15 +38225,31 @@
           <t>SNEL</t>
         </is>
       </c>
-      <c r="F832" s="2" t="n"/>
-      <c r="G832" s="2" t="n"/>
-      <c r="H832" s="2" t="n"/>
-      <c r="I832" s="2" t="n"/>
+      <c r="F832" s="2" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="G832" s="2" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H832" s="2" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="I832" s="2" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
     </row>
     <row r="833">
       <c r="A833" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B833" s="2" t="inlineStr">
@@ -37555,7 +38259,7 @@
       </c>
       <c r="C833" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Énergie</t>
         </is>
       </c>
       <c r="D833" s="2" t="inlineStr">
@@ -37563,10 +38267,26 @@
           <t>ZESCO</t>
         </is>
       </c>
-      <c r="F833" s="2" t="n"/>
-      <c r="G833" s="2" t="n"/>
-      <c r="H833" s="2" t="n"/>
-      <c r="I833" s="2" t="n"/>
+      <c r="F833" s="2" t="inlineStr">
+        <is>
+          <t>Mid cap 200M-1Md</t>
+        </is>
+      </c>
+      <c r="G833" s="2" t="inlineStr">
+        <is>
+          <t>ZMW 30.8 Md</t>
+        </is>
+      </c>
+      <c r="H833" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I833" s="2" t="inlineStr">
+        <is>
+          <t>https://diggers.news/business/2025/12/29/zescos-turnover-increased-to-k30-8-billion-in-2024-report/</t>
+        </is>
+      </c>
     </row>
     <row r="834">
       <c r="A834" s="5" t="inlineStr">
@@ -40721,7 +41441,7 @@
     <row r="909">
       <c r="A909" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Non</t>
         </is>
       </c>
       <c r="B909" s="2" t="inlineStr">
@@ -40739,15 +41459,31 @@
           <t>IREN</t>
         </is>
       </c>
-      <c r="F909" s="2" t="n"/>
-      <c r="G909" s="2" t="n"/>
-      <c r="H909" s="2" t="n"/>
-      <c r="I909" s="2" t="n"/>
+      <c r="F909" s="2" t="inlineStr">
+        <is>
+          <t>Small cap &lt;200M</t>
+        </is>
+      </c>
+      <c r="G909" s="2" t="inlineStr">
+        <is>
+          <t>USD 184.1 M</t>
+        </is>
+      </c>
+      <c r="H909" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I909" s="2" t="inlineStr">
+        <is>
+          <t>https://iren.com/investors/reports</t>
+        </is>
+      </c>
     </row>
     <row r="910">
       <c r="A910" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B910" s="2" t="inlineStr">
@@ -40757,7 +41493,7 @@
       </c>
       <c r="C910" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Énergie</t>
         </is>
       </c>
       <c r="D910" s="2" t="inlineStr">
@@ -40765,15 +41501,31 @@
           <t>AGL Energy</t>
         </is>
       </c>
-      <c r="F910" s="2" t="n"/>
-      <c r="G910" s="2" t="n"/>
-      <c r="H910" s="2" t="n"/>
-      <c r="I910" s="2" t="n"/>
+      <c r="F910" s="2" t="inlineStr">
+        <is>
+          <t>Large cap / groupe &gt;1 Md</t>
+        </is>
+      </c>
+      <c r="G910" s="2" t="inlineStr">
+        <is>
+          <t>AUD 13.6 Md</t>
+        </is>
+      </c>
+      <c r="H910" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I910" s="2" t="inlineStr">
+        <is>
+          <t>https://stockanalysis.com/quote/asx/AGL/revenue/</t>
+        </is>
+      </c>
     </row>
     <row r="911">
       <c r="A911" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B911" s="2" t="inlineStr">
@@ -40783,7 +41535,7 @@
       </c>
       <c r="C911" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Énergie</t>
         </is>
       </c>
       <c r="D911" s="2" t="inlineStr">
@@ -40791,15 +41543,31 @@
           <t>Origin Energy</t>
         </is>
       </c>
-      <c r="F911" s="2" t="n"/>
-      <c r="G911" s="2" t="n"/>
-      <c r="H911" s="2" t="n"/>
-      <c r="I911" s="2" t="n"/>
+      <c r="F911" s="2" t="inlineStr">
+        <is>
+          <t>Large cap / groupe &gt;1 Md</t>
+        </is>
+      </c>
+      <c r="G911" s="2" t="inlineStr">
+        <is>
+          <t>AUD 16.18 Md</t>
+        </is>
+      </c>
+      <c r="H911" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I911" s="2" t="inlineStr">
+        <is>
+          <t>https://stockanalysis.com/quote/otc/OGFGF/revenue/</t>
+        </is>
+      </c>
     </row>
     <row r="912">
       <c r="A912" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B912" s="2" t="inlineStr">
@@ -40809,7 +41577,7 @@
       </c>
       <c r="C912" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Énergie</t>
         </is>
       </c>
       <c r="D912" s="2" t="inlineStr">
@@ -40817,15 +41585,31 @@
           <t>EnergyAustralia</t>
         </is>
       </c>
-      <c r="F912" s="2" t="n"/>
-      <c r="G912" s="2" t="n"/>
-      <c r="H912" s="2" t="n"/>
-      <c r="I912" s="2" t="n"/>
+      <c r="F912" s="2" t="inlineStr">
+        <is>
+          <t>Large cap / groupe &gt;1 Md</t>
+        </is>
+      </c>
+      <c r="G912" s="2" t="inlineStr">
+        <is>
+          <t>AUD 7 197 M</t>
+        </is>
+      </c>
+      <c r="H912" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I912" s="2" t="inlineStr">
+        <is>
+          <t>https://www.energyaustralia.com.au/about-us/media/news/energyaustralia-delivers-improved-performance</t>
+        </is>
+      </c>
     </row>
     <row r="913">
       <c r="A913" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B913" s="2" t="inlineStr">
@@ -40835,7 +41619,7 @@
       </c>
       <c r="C913" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Énergie</t>
         </is>
       </c>
       <c r="D913" s="2" t="inlineStr">
@@ -40843,15 +41627,31 @@
           <t>Meridian Energy</t>
         </is>
       </c>
-      <c r="F913" s="2" t="n"/>
-      <c r="G913" s="2" t="n"/>
-      <c r="H913" s="2" t="n"/>
-      <c r="I913" s="2" t="n"/>
+      <c r="F913" s="2" t="inlineStr">
+        <is>
+          <t>Large cap / groupe &gt;1 Md</t>
+        </is>
+      </c>
+      <c r="G913" s="2" t="inlineStr">
+        <is>
+          <t>NZD 4.86 Md</t>
+        </is>
+      </c>
+      <c r="H913" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I913" s="2" t="inlineStr">
+        <is>
+          <t>https://www.meridianenergy.co.nz/about-us/investors/reports/annual-results-and-reports</t>
+        </is>
+      </c>
     </row>
     <row r="914">
       <c r="A914" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B914" s="2" t="inlineStr">
@@ -40861,7 +41661,7 @@
       </c>
       <c r="C914" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Énergie</t>
         </is>
       </c>
       <c r="D914" s="2" t="inlineStr">
@@ -40869,15 +41669,31 @@
           <t>Contact Energy</t>
         </is>
       </c>
-      <c r="F914" s="2" t="n"/>
-      <c r="G914" s="2" t="n"/>
-      <c r="H914" s="2" t="n"/>
-      <c r="I914" s="2" t="n"/>
+      <c r="F914" s="2" t="inlineStr">
+        <is>
+          <t>Large cap / groupe &gt;1 Md</t>
+        </is>
+      </c>
+      <c r="G914" s="2" t="inlineStr">
+        <is>
+          <t>NZD 2.87 Md</t>
+        </is>
+      </c>
+      <c r="H914" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I914" s="2" t="inlineStr">
+        <is>
+          <t>https://companiesmarketcap.com/nzd/contact-energy/revenue/</t>
+        </is>
+      </c>
     </row>
     <row r="915">
       <c r="A915" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B915" s="2" t="inlineStr">
@@ -40887,7 +41703,7 @@
       </c>
       <c r="C915" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Énergie</t>
         </is>
       </c>
       <c r="D915" s="2" t="inlineStr">
@@ -40895,15 +41711,31 @@
           <t>Genesis Energy</t>
         </is>
       </c>
-      <c r="F915" s="2" t="n"/>
-      <c r="G915" s="2" t="n"/>
-      <c r="H915" s="2" t="n"/>
-      <c r="I915" s="2" t="n"/>
+      <c r="F915" s="2" t="inlineStr">
+        <is>
+          <t>Large cap / groupe &gt;1 Md</t>
+        </is>
+      </c>
+      <c r="G915" s="2" t="inlineStr">
+        <is>
+          <t>NZD 2.62 Md</t>
+        </is>
+      </c>
+      <c r="H915" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I915" s="2" t="inlineStr">
+        <is>
+          <t>https://companiesmarketcap.com/nzd/genesis-energy/revenue/</t>
+        </is>
+      </c>
     </row>
     <row r="916">
       <c r="A916" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B916" s="2" t="inlineStr">
@@ -40913,7 +41745,7 @@
       </c>
       <c r="C916" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Énergie</t>
         </is>
       </c>
       <c r="D916" s="2" t="inlineStr">
@@ -40921,15 +41753,31 @@
           <t>Mercury NZ</t>
         </is>
       </c>
-      <c r="F916" s="2" t="n"/>
-      <c r="G916" s="2" t="n"/>
-      <c r="H916" s="2" t="n"/>
-      <c r="I916" s="2" t="n"/>
+      <c r="F916" s="2" t="inlineStr">
+        <is>
+          <t>Large cap / groupe &gt;1 Md</t>
+        </is>
+      </c>
+      <c r="G916" s="2" t="inlineStr">
+        <is>
+          <t>NZD 3.43 Md</t>
+        </is>
+      </c>
+      <c r="H916" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I916" s="2" t="inlineStr">
+        <is>
+          <t>https://www.listcorp.com/asx/mcy/mercury-nz-limited/news/fy2024-full-year-results-3070818.html</t>
+        </is>
+      </c>
     </row>
     <row r="917">
       <c r="A917" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B917" s="2" t="inlineStr">
@@ -40939,7 +41787,7 @@
       </c>
       <c r="C917" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Énergie</t>
         </is>
       </c>
       <c r="D917" s="2" t="inlineStr">
@@ -40947,15 +41795,31 @@
           <t>Infratil</t>
         </is>
       </c>
-      <c r="F917" s="2" t="n"/>
-      <c r="G917" s="2" t="n"/>
-      <c r="H917" s="2" t="n"/>
-      <c r="I917" s="2" t="n"/>
+      <c r="F917" s="2" t="inlineStr">
+        <is>
+          <t>Large cap / groupe &gt;1 Md</t>
+        </is>
+      </c>
+      <c r="G917" s="2" t="inlineStr">
+        <is>
+          <t>NZD 3.24 Md</t>
+        </is>
+      </c>
+      <c r="H917" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I917" s="2" t="inlineStr">
+        <is>
+          <t>https://infratil.com/news/infratil-full-year-results-for-the-year-ended-31-march-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="918">
       <c r="A918" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B918" s="2" t="inlineStr">
@@ -40965,7 +41829,7 @@
       </c>
       <c r="C918" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Énergie</t>
         </is>
       </c>
       <c r="D918" s="2" t="inlineStr">
@@ -40973,15 +41837,31 @@
           <t>APA Group</t>
         </is>
       </c>
-      <c r="F918" s="2" t="n"/>
-      <c r="G918" s="2" t="n"/>
-      <c r="H918" s="2" t="n"/>
-      <c r="I918" s="2" t="n"/>
+      <c r="F918" s="2" t="inlineStr">
+        <is>
+          <t>Large cap / groupe &gt;1 Md</t>
+        </is>
+      </c>
+      <c r="G918" s="2" t="inlineStr">
+        <is>
+          <t>AUD 3.06 Md</t>
+        </is>
+      </c>
+      <c r="H918" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I918" s="2" t="inlineStr">
+        <is>
+          <t>https://stockanalysis.com/quote/asx/APA/revenue/</t>
+        </is>
+      </c>
     </row>
     <row r="919">
       <c r="A919" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B919" s="2" t="inlineStr">
@@ -40991,7 +41871,7 @@
       </c>
       <c r="C919" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Data center / télécom / Software</t>
         </is>
       </c>
       <c r="D919" s="2" t="inlineStr">
@@ -40999,15 +41879,31 @@
           <t>NEXTDC</t>
         </is>
       </c>
-      <c r="F919" s="2" t="n"/>
-      <c r="G919" s="2" t="n"/>
-      <c r="H919" s="2" t="n"/>
-      <c r="I919" s="2" t="n"/>
+      <c r="F919" s="2" t="inlineStr">
+        <is>
+          <t>Mid cap 200M-1Md</t>
+        </is>
+      </c>
+      <c r="G919" s="2" t="inlineStr">
+        <is>
+          <t>AUD 404.3 M</t>
+        </is>
+      </c>
+      <c r="H919" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I919" s="2" t="inlineStr">
+        <is>
+          <t>https://nextdc.com/hubfs/Financial%20Reports/280827%20-%20FY24%20Results%20Announcement.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="920" ht="24" customHeight="1">
       <c r="A920" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B920" s="2" t="inlineStr">
@@ -41017,7 +41913,7 @@
       </c>
       <c r="C920" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Data center / télécom / Software</t>
         </is>
       </c>
       <c r="D920" s="2" t="inlineStr">
@@ -41025,15 +41921,31 @@
           <t>Macquarie Technology Group</t>
         </is>
       </c>
-      <c r="F920" s="2" t="n"/>
-      <c r="G920" s="2" t="n"/>
-      <c r="H920" s="2" t="n"/>
-      <c r="I920" s="2" t="n"/>
+      <c r="F920" s="2" t="inlineStr">
+        <is>
+          <t>Mid cap 200M-1Md</t>
+        </is>
+      </c>
+      <c r="G920" s="2" t="inlineStr">
+        <is>
+          <t>AUD 363.3 M</t>
+        </is>
+      </c>
+      <c r="H920" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I920" s="2" t="inlineStr">
+        <is>
+          <t>https://www.macquarietechnologygroup.com/assets/wp-content/uploads/2024/09/MAQ-2024-Appendix-4E-Annual-Report.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="921">
       <c r="A921" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B921" s="2" t="inlineStr">
@@ -41043,7 +41955,7 @@
       </c>
       <c r="C921" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Data center / télécom / Software</t>
         </is>
       </c>
       <c r="D921" s="2" t="inlineStr">
@@ -41051,15 +41963,31 @@
           <t>Superloop</t>
         </is>
       </c>
-      <c r="F921" s="2" t="n"/>
-      <c r="G921" s="2" t="n"/>
-      <c r="H921" s="2" t="n"/>
-      <c r="I921" s="2" t="n"/>
+      <c r="F921" s="2" t="inlineStr">
+        <is>
+          <t>Mid cap 200M-1Md</t>
+        </is>
+      </c>
+      <c r="G921" s="2" t="inlineStr">
+        <is>
+          <t>AUD 416.6 M</t>
+        </is>
+      </c>
+      <c r="H921" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I921" s="2" t="inlineStr">
+        <is>
+          <t>https://stockanalysis.com/quote/asx/SLC/revenue/</t>
+        </is>
+      </c>
     </row>
     <row r="922">
       <c r="A922" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B922" s="2" t="inlineStr">
@@ -41069,7 +41997,7 @@
       </c>
       <c r="C922" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Data center / télécom / Software</t>
         </is>
       </c>
       <c r="D922" s="2" t="inlineStr">
@@ -41077,15 +42005,31 @@
           <t>Spark New Zealand</t>
         </is>
       </c>
-      <c r="F922" s="2" t="n"/>
-      <c r="G922" s="2" t="n"/>
-      <c r="H922" s="2" t="n"/>
-      <c r="I922" s="2" t="n"/>
+      <c r="F922" s="2" t="inlineStr">
+        <is>
+          <t>Large cap / groupe &gt;1 Md</t>
+        </is>
+      </c>
+      <c r="G922" s="2" t="inlineStr">
+        <is>
+          <t>NZD 3.86 Md</t>
+        </is>
+      </c>
+      <c r="H922" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I922" s="2" t="inlineStr">
+        <is>
+          <t>https://uk.marketscreener.com/quote/stock/SPARK-NEW-ZEALAND-LIMITED-6492600/news/Spark-New-Zealand-Posts-Fiscal-2024-Revenue-Down-14-to-NZ-3-86-Billion-EPS-of-NZ-0-173-47716076/</t>
+        </is>
+      </c>
     </row>
     <row r="923">
       <c r="A923" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A verifier </t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="B923" s="2" t="inlineStr">
@@ -41095,7 +42039,7 @@
       </c>
       <c r="C923" s="2" t="inlineStr">
         <is>
-          <t>Crypto mining</t>
+          <t>Data center / télécom / Software</t>
         </is>
       </c>
       <c r="D923" s="2" t="inlineStr">
@@ -41103,10 +42047,26 @@
           <t>Telstra</t>
         </is>
       </c>
-      <c r="F923" s="2" t="n"/>
-      <c r="G923" s="2" t="n"/>
-      <c r="H923" s="2" t="n"/>
-      <c r="I923" s="2" t="n"/>
+      <c r="F923" s="2" t="inlineStr">
+        <is>
+          <t>Large cap / groupe &gt;1 Md</t>
+        </is>
+      </c>
+      <c r="G923" s="2" t="inlineStr">
+        <is>
+          <t>AUD 23.5 Md</t>
+        </is>
+      </c>
+      <c r="H923" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I923" s="2" t="inlineStr">
+        <is>
+          <t>https://www.telstra.com.au/content/dam/tcom/about-us/investors/pdf-g/telstra-annual-report-2024-interactive.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="924">
       <c r="A924" s="5" t="inlineStr">

</xml_diff>